<commit_message>
update test reports 2026-05-22 00:02:33
</commit_message>
<xml_diff>
--- a/Web Dashboard/Configuration Group/Add Configuration Group/configuration_group.xlsx
+++ b/Web Dashboard/Configuration Group/Add Configuration Group/configuration_group.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25726"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED70FFB6-D9D6-49CD-A4B3-82C4254FEC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Test Cases" state="visible" r:id="rId4"/>
+    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -112,7 +113,7 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>21/5/2026, 15.14.54</t>
+    <t>13/5/2026, 14.23.42</t>
   </si>
   <si>
     <t>CO-002</t>
@@ -133,7 +134,7 @@
     <t>Expected text not found on page: "Status must be filled. Please fill status"</t>
   </si>
   <si>
-    <t>21/5/2026, 15.15.04</t>
+    <t>13/5/2026, 14.23.53</t>
   </si>
   <si>
     <t>CO-003</t>
@@ -148,13 +149,13 @@
     <t>Settings must be filled</t>
   </si>
   <si>
-    <t>21/5/2026, 15.15.13</t>
+    <t>13/5/2026, 14.24.02</t>
   </si>
   <si>
     <t>CO-004</t>
   </si>
   <si>
-    <t>21/5/2026, 15.15.20</t>
+    <t>13/5/2026, 14.24.08</t>
   </si>
   <si>
     <t>CO-005</t>
@@ -169,41 +170,43 @@
     <t>Open Loop Active - KYC Only settings</t>
   </si>
   <si>
-    <t>21/5/2026, 15.15.25</t>
+    <t>13/5/2026, 14.24.13</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <color rgb="FFCC0000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFCC0000"/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
       <color rgb="FF006600"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -595,9 +598,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T6"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
@@ -616,7 +619,7 @@
     <col min="20" max="20" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -978,6 +981,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>